<commit_message>
updated fig doc and sasprogram
</commit_message>
<xml_diff>
--- a/bankole_2026/documentation/figures_11amm.xlsx
+++ b/bankole_2026/documentation/figures_11amm.xlsx
@@ -86,10 +86,10 @@
   </si>
   <si>
     <t xml:space="preserve">creates tables used for ribbon plots
-Creates supp table 4</t>
-  </si>
-  <si>
-    <t xml:space="preserve">count_for_flow_chart_07lmm.sas</t>
+Creates supp table 4 and 1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">count_for_flow_chart_11lmm.sas</t>
   </si>
   <si>
     <t xml:space="preserve">PROJ/submission/supplementary/
@@ -103,9 +103,9 @@
 /Tables/merged_fiveSpecies_component_summary.csv (now component summary in zendo)</t>
   </si>
   <si>
-    <t xml:space="preserve">McIntyre_Lab/sex_specific_splicing/Tables/count_origin_anno_xpress.csv (sup table4)
-McIntyre_Lab/sex_specific_splicing/Tables/count_origin_anno_xpress_byspecies.csv
-PROJ/submission/supplementary/fiveSpecies_annotations/link_files/component_info.csv
+    <t xml:space="preserve">McIntyre_Lab/sex_specific_splicing/Tables/count_origin_anno_xpress.csv (sup table1)
+McIntyre_Lab/sex_specific_splicing/Tables/count_origin_anno_xpress_byspecies.csv (ST4)
+PROJ/Tables/component_info.csv
 PROJ//Tables/count_components_expressed_by_category.csv
 PROJ/Tables/cnt_mel_sim_sex.csv
 PROJ/Tables/cnt_mel_sim_ser_sex.csv"
@@ -797,6 +797,7 @@
       <sz val="10"/>
       <name val="Arial"/>
       <family val="2"/>
+      <charset val="1"/>
     </font>
     <font>
       <sz val="10"/>
@@ -819,6 +820,7 @@
       <sz val="10"/>
       <name val="Arial"/>
       <family val="2"/>
+      <charset val="1"/>
     </font>
   </fonts>
   <fills count="4">
@@ -875,7 +877,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="10">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -914,14 +916,6 @@
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
   </cellXfs>
@@ -1110,8 +1104,7 @@
   <dimension ref="B1:H56"/>
   <sheetFormatPr defaultColWidth="11.5625" defaultRowHeight="12.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="23"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="23"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="1" style="1" width="23"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="2" width="47.67"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="4" style="1" width="34.33"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="45.22"/>
@@ -1194,7 +1187,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="14" customFormat="false" ht="258.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="14" customFormat="false" ht="281.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B14" s="6" t="s">
         <v>20</v>
       </c>
@@ -1208,14 +1201,14 @@
       <c r="F14" s="7" t="s">
         <v>23</v>
       </c>
-      <c r="G14" s="2" t="s">
+      <c r="G14" s="9" t="s">
         <v>24</v>
       </c>
       <c r="H14" s="6" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="15" customFormat="false" ht="326.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="15" customFormat="false" ht="326.1" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B15" s="2" t="s">
         <v>26</v>
       </c>
@@ -1231,7 +1224,7 @@
       <c r="G15" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="H15" s="9" t="s">
+      <c r="H15" s="7" t="s">
         <v>31</v>
       </c>
     </row>
@@ -1240,11 +1233,11 @@
       <c r="F16" s="2"/>
       <c r="G16" s="2"/>
     </row>
-    <row r="17" customFormat="false" ht="147.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="17" customFormat="false" ht="135.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B17" s="2" t="s">
         <v>32</v>
       </c>
-      <c r="C17" s="9" t="s">
+      <c r="C17" s="7" t="s">
         <v>33</v>
       </c>
       <c r="D17" s="2" t="s">
@@ -1253,11 +1246,11 @@
       <c r="G17" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="H17" s="9" t="s">
+      <c r="H17" s="7" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="19" customFormat="false" ht="304.1" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="19" customFormat="false" ht="292.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B19" s="2" t="s">
         <v>37</v>
       </c>
@@ -1273,7 +1266,7 @@
       <c r="G19" s="2" t="s">
         <v>41</v>
       </c>
-      <c r="H19" s="9" t="s">
+      <c r="H19" s="7" t="s">
         <v>42</v>
       </c>
     </row>
@@ -1284,7 +1277,7 @@
       <c r="C21" s="2" t="s">
         <v>44</v>
       </c>
-      <c r="D21" s="10" t="s">
+      <c r="D21" s="8" t="s">
         <v>45</v>
       </c>
       <c r="F21" s="2" t="s">
@@ -1293,7 +1286,7 @@
       <c r="G21" s="2" t="s">
         <v>47</v>
       </c>
-      <c r="H21" s="9" t="s">
+      <c r="H21" s="7" t="s">
         <v>48</v>
       </c>
     </row>
@@ -1304,7 +1297,7 @@
       <c r="C23" s="2" t="s">
         <v>50</v>
       </c>
-      <c r="D23" s="10" t="s">
+      <c r="D23" s="8" t="s">
         <v>51</v>
       </c>
       <c r="F23" s="2" t="s">
@@ -1313,7 +1306,7 @@
       <c r="G23" s="2" t="s">
         <v>53</v>
       </c>
-      <c r="H23" s="9"/>
+      <c r="H23" s="7"/>
     </row>
     <row r="25" customFormat="false" ht="135.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B25" s="2" t="s">
@@ -1322,7 +1315,7 @@
       <c r="C25" s="2" t="s">
         <v>55</v>
       </c>
-      <c r="D25" s="10" t="s">
+      <c r="D25" s="8" t="s">
         <v>56</v>
       </c>
       <c r="F25" s="2" t="s">
@@ -1331,7 +1324,7 @@
       <c r="G25" s="2" t="s">
         <v>57</v>
       </c>
-      <c r="H25" s="9" t="s">
+      <c r="H25" s="7" t="s">
         <v>58</v>
       </c>
     </row>
@@ -1355,7 +1348,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="29" customFormat="false" ht="214.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="29" customFormat="false" ht="214.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B29" s="2" t="s">
         <v>65</v>
       </c>
@@ -1375,7 +1368,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="31" customFormat="false" ht="102.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="31" customFormat="false" ht="79.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B31" s="2" t="s">
         <v>71</v>
       </c>
@@ -1388,14 +1381,14 @@
       <c r="F31" s="2" t="s">
         <v>74</v>
       </c>
-      <c r="G31" s="10" t="s">
+      <c r="G31" s="8" t="s">
         <v>75</v>
       </c>
-      <c r="H31" s="9" t="s">
+      <c r="H31" s="7" t="s">
         <v>76</v>
       </c>
     </row>
-    <row r="33" customFormat="false" ht="192.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="33" customFormat="false" ht="180.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B33" s="2" t="s">
         <v>77</v>
       </c>
@@ -1433,70 +1426,69 @@
         <v>87</v>
       </c>
     </row>
-    <row r="37" s="11" customFormat="true" ht="281.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="37" s="1" customFormat="true" ht="281.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B37" s="1" t="s">
         <v>88</v>
       </c>
-      <c r="C37" s="9" t="s">
+      <c r="C37" s="7" t="s">
         <v>89</v>
       </c>
-      <c r="D37" s="10" t="s">
+      <c r="D37" s="8" t="s">
         <v>90</v>
       </c>
-      <c r="E37" s="1"/>
       <c r="F37" s="1" t="s">
         <v>86</v>
       </c>
-      <c r="G37" s="10" t="s">
+      <c r="G37" s="8" t="s">
         <v>91</v>
       </c>
-      <c r="H37" s="9" t="s">
+      <c r="H37" s="7" t="s">
         <v>92</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C38" s="1"/>
     </row>
-    <row r="39" customFormat="false" ht="192.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="39" customFormat="false" ht="191.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B39" s="2" t="s">
         <v>93</v>
       </c>
       <c r="C39" s="2" t="s">
         <v>94</v>
       </c>
-      <c r="D39" s="10" t="s">
+      <c r="D39" s="8" t="s">
         <v>95</v>
       </c>
       <c r="F39" s="2" t="s">
         <v>96</v>
       </c>
-      <c r="G39" s="10" t="s">
+      <c r="G39" s="8" t="s">
         <v>97</v>
       </c>
-      <c r="H39" s="9" t="s">
+      <c r="H39" s="7" t="s">
         <v>98</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C40" s="1"/>
     </row>
-    <row r="41" customFormat="false" ht="494.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="41" customFormat="false" ht="494" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B41" s="2" t="s">
         <v>99</v>
       </c>
       <c r="C41" s="2" t="s">
         <v>100</v>
       </c>
-      <c r="D41" s="10" t="s">
+      <c r="D41" s="8" t="s">
         <v>101</v>
       </c>
       <c r="F41" s="2" t="s">
         <v>102</v>
       </c>
-      <c r="G41" s="10" t="s">
+      <c r="G41" s="8" t="s">
         <v>103</v>
       </c>
-      <c r="H41" s="9" t="s">
+      <c r="H41" s="7" t="s">
         <v>104</v>
       </c>
     </row>
@@ -1504,32 +1496,32 @@
       <c r="C42" s="1"/>
     </row>
     <row r="43" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B43" s="9" t="s">
+      <c r="B43" s="7" t="s">
         <v>105</v>
       </c>
       <c r="C43" s="1"/>
-      <c r="D43" s="9" t="s">
+      <c r="D43" s="7" t="s">
         <v>106</v>
       </c>
-      <c r="F43" s="9" t="s">
+      <c r="F43" s="7" t="s">
         <v>107</v>
       </c>
-      <c r="G43" s="9" t="s">
+      <c r="G43" s="7" t="s">
         <v>108</v>
       </c>
-      <c r="H43" s="9"/>
+      <c r="H43" s="7"/>
     </row>
     <row r="44" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C44" s="1"/>
     </row>
-    <row r="45" customFormat="false" ht="214.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="45" customFormat="false" ht="202.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B45" s="2" t="s">
         <v>109</v>
       </c>
-      <c r="C45" s="9" t="s">
+      <c r="C45" s="7" t="s">
         <v>110</v>
       </c>
-      <c r="D45" s="10" t="s">
+      <c r="D45" s="8" t="s">
         <v>111</v>
       </c>
       <c r="F45" s="2" t="s">
@@ -1538,7 +1530,7 @@
       <c r="G45" s="2" t="s">
         <v>113</v>
       </c>
-      <c r="H45" s="9" t="s">
+      <c r="H45" s="7" t="s">
         <v>114</v>
       </c>
     </row>
@@ -1600,7 +1592,7 @@
       <c r="C53" s="2" t="s">
         <v>130</v>
       </c>
-      <c r="D53" s="10" t="s">
+      <c r="D53" s="8" t="s">
         <v>131</v>
       </c>
       <c r="H53" s="2" t="s">
@@ -1611,7 +1603,7 @@
       <c r="B54" s="2" t="s">
         <v>133</v>
       </c>
-      <c r="D54" s="10" t="s">
+      <c r="D54" s="8" t="s">
         <v>131</v>
       </c>
       <c r="H54" s="2" t="s">
@@ -1625,7 +1617,7 @@
       <c r="C56" s="2" t="s">
         <v>136</v>
       </c>
-      <c r="D56" s="10" t="s">
+      <c r="D56" s="8" t="s">
         <v>137</v>
       </c>
       <c r="F56" s="2" t="s">

</xml_diff>